<commit_message>
Atividade 10 - parte 4
</commit_message>
<xml_diff>
--- a/Avancado/10 - Ferramentas de Base de Dados.xlsx
+++ b/Avancado/10 - Ferramentas de Base de Dados.xlsx
@@ -1,32 +1,44 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilck.alunos\Desktop\EXCEL-completo\Avancado\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luizh\Excel completo SENAI\Avancado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22F6441D-BB68-43E3-8D3A-B668F5785211}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5BF9B02-49AC-41FC-B7D8-8892C7CAE731}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Base de Dados" sheetId="1" r:id="rId1"/>
     <sheet name="Subtotal" sheetId="2" r:id="rId2"/>
+    <sheet name="Filtro avançado" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="179021"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="63">
   <si>
     <t>NOME</t>
   </si>
@@ -191,6 +203,30 @@
   </si>
   <si>
     <t>Total Geral</t>
+  </si>
+  <si>
+    <t>Área de critérios</t>
+  </si>
+  <si>
+    <t>Área de extração</t>
+  </si>
+  <si>
+    <t>RESUMO</t>
+  </si>
+  <si>
+    <t>BDSOMA</t>
+  </si>
+  <si>
+    <t>BDMÉDIA</t>
+  </si>
+  <si>
+    <t>BDMIN</t>
+  </si>
+  <si>
+    <t>BDMÁX</t>
+  </si>
+  <si>
+    <t>BDCONTAR</t>
   </si>
 </sst>
 </file>
@@ -199,7 +235,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="166" formatCode="&quot;R$&quot;\ #,##0.00"/>
+    <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -225,7 +261,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -235,6 +271,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -295,7 +343,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -327,16 +375,36 @@
     <xf numFmtId="44" fontId="2" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
@@ -619,20 +687,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.44140625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -661,7 +729,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>17</v>
       </c>
@@ -688,7 +756,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>18</v>
       </c>
@@ -719,7 +787,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>19</v>
       </c>
@@ -750,7 +818,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
@@ -781,7 +849,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>21</v>
       </c>
@@ -812,7 +880,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>22</v>
       </c>
@@ -843,7 +911,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>23</v>
       </c>
@@ -874,7 +942,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>24</v>
       </c>
@@ -901,7 +969,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>25</v>
       </c>
@@ -932,7 +1000,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>26</v>
       </c>
@@ -963,7 +1031,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>27</v>
       </c>
@@ -994,7 +1062,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>28</v>
       </c>
@@ -1025,7 +1093,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>29</v>
       </c>
@@ -1052,7 +1120,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>30</v>
       </c>
@@ -1083,7 +1151,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>31</v>
       </c>
@@ -1114,7 +1182,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
@@ -1145,7 +1213,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>33</v>
       </c>
@@ -1172,7 +1240,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>34</v>
       </c>
@@ -1203,7 +1271,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>35</v>
       </c>
@@ -1234,7 +1302,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>36</v>
       </c>
@@ -1265,7 +1333,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>37</v>
       </c>
@@ -1292,7 +1360,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>38</v>
       </c>
@@ -1323,7 +1391,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>39</v>
       </c>
@@ -1354,7 +1422,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>40</v>
       </c>
@@ -1385,7 +1453,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>41</v>
       </c>
@@ -1412,7 +1480,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>42</v>
       </c>
@@ -1443,7 +1511,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>43</v>
       </c>
@@ -1474,7 +1542,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>44</v>
       </c>
@@ -1505,7 +1573,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>45</v>
       </c>
@@ -1536,7 +1604,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>46</v>
       </c>
@@ -1563,7 +1631,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>47</v>
       </c>
@@ -1594,7 +1662,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>48</v>
       </c>
@@ -1625,7 +1693,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>49</v>
       </c>
@@ -1652,7 +1720,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>50</v>
       </c>
@@ -1692,19 +1760,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8731D695-52D1-48A5-99CD-9023713EAF57}">
   <dimension ref="A1:I39"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="14.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -1733,7 +1801,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>23</v>
       </c>
@@ -1750,11 +1818,11 @@
         <v>611.82000000000005</v>
       </c>
       <c r="F2" s="9" t="str">
-        <f>_xlfn.IFS(D2="","NÃO CONSTA", D2&lt;=C2,"PAGO", D2&gt;C2,"ATRASO")</f>
+        <f t="shared" ref="F2:F13" si="0">_xlfn.IFS(D2="","NÃO CONSTA", D2&lt;=C2,"PAGO", D2&gt;C2,"ATRASO")</f>
         <v>ATRASO</v>
       </c>
       <c r="G2" s="9">
-        <f>IF(D2&lt;=C2,0,_xlfn.DAYS(D2,C2))</f>
+        <f t="shared" ref="G2:G13" si="1">IF(D2&lt;=C2,0,_xlfn.DAYS(D2,C2))</f>
         <v>1</v>
       </c>
       <c r="H2" s="9" t="s">
@@ -1764,7 +1832,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>25</v>
       </c>
@@ -1781,11 +1849,11 @@
         <v>633.63</v>
       </c>
       <c r="F3" s="2" t="str">
-        <f>_xlfn.IFS(D3="","NÃO CONSTA", D3&lt;=C3,"PAGO", D3&gt;C3,"ATRASO")</f>
+        <f t="shared" si="0"/>
         <v>ATRASO</v>
       </c>
       <c r="G3" s="2">
-        <f>IF(D3&lt;=C3,0,_xlfn.DAYS(D3,C3))</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="H3" s="2" t="s">
@@ -1795,7 +1863,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>26</v>
       </c>
@@ -1812,11 +1880,11 @@
         <v>633.63</v>
       </c>
       <c r="F4" s="2" t="str">
-        <f>_xlfn.IFS(D4="","NÃO CONSTA", D4&lt;=C4,"PAGO", D4&gt;C4,"ATRASO")</f>
+        <f t="shared" si="0"/>
         <v>ATRASO</v>
       </c>
       <c r="G4" s="2">
-        <f>IF(D4&lt;=C4,0,_xlfn.DAYS(D4,C4))</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="H4" s="2" t="s">
@@ -1826,7 +1894,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>27</v>
       </c>
@@ -1843,11 +1911,11 @@
         <v>700</v>
       </c>
       <c r="F5" s="2" t="str">
-        <f>_xlfn.IFS(D5="","NÃO CONSTA", D5&lt;=C5,"PAGO", D5&gt;C5,"ATRASO")</f>
+        <f t="shared" si="0"/>
         <v>ATRASO</v>
       </c>
       <c r="G5" s="2">
-        <f>IF(D5&lt;=C5,0,_xlfn.DAYS(D5,C5))</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="H5" s="2" t="s">
@@ -1857,7 +1925,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>28</v>
       </c>
@@ -1874,11 +1942,11 @@
         <v>733.37</v>
       </c>
       <c r="F6" s="2" t="str">
-        <f>_xlfn.IFS(D6="","NÃO CONSTA", D6&lt;=C6,"PAGO", D6&gt;C6,"ATRASO")</f>
+        <f t="shared" si="0"/>
         <v>ATRASO</v>
       </c>
       <c r="G6" s="2">
-        <f>IF(D6&lt;=C6,0,_xlfn.DAYS(D6,C6))</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="H6" s="2" t="s">
@@ -1888,7 +1956,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>30</v>
       </c>
@@ -1905,11 +1973,11 @@
         <v>733.37</v>
       </c>
       <c r="F7" s="2" t="str">
-        <f>_xlfn.IFS(D7="","NÃO CONSTA", D7&lt;=C7,"PAGO", D7&gt;C7,"ATRASO")</f>
+        <f t="shared" si="0"/>
         <v>ATRASO</v>
       </c>
       <c r="G7" s="2">
-        <f>IF(D7&lt;=C7,0,_xlfn.DAYS(D7,C7))</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="H7" s="2" t="s">
@@ -1919,7 +1987,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>36</v>
       </c>
@@ -1936,11 +2004,11 @@
         <v>815.3</v>
       </c>
       <c r="F8" s="2" t="str">
-        <f>_xlfn.IFS(D8="","NÃO CONSTA", D8&lt;=C8,"PAGO", D8&gt;C8,"ATRASO")</f>
+        <f t="shared" si="0"/>
         <v>ATRASO</v>
       </c>
       <c r="G8" s="2">
-        <f>IF(D8&lt;=C8,0,_xlfn.DAYS(D8,C8))</f>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="H8" s="2" t="s">
@@ -1950,7 +2018,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>38</v>
       </c>
@@ -1967,11 +2035,11 @@
         <v>841.37</v>
       </c>
       <c r="F9" s="2" t="str">
-        <f>_xlfn.IFS(D9="","NÃO CONSTA", D9&lt;=C9,"PAGO", D9&gt;C9,"ATRASO")</f>
+        <f t="shared" si="0"/>
         <v>ATRASO</v>
       </c>
       <c r="G9" s="2">
-        <f>IF(D9&lt;=C9,0,_xlfn.DAYS(D9,C9))</f>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="H9" s="2" t="s">
@@ -1981,7 +2049,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>39</v>
       </c>
@@ -1998,11 +2066,11 @@
         <v>841.37</v>
       </c>
       <c r="F10" s="2" t="str">
-        <f>_xlfn.IFS(D10="","NÃO CONSTA", D10&lt;=C10,"PAGO", D10&gt;C10,"ATRASO")</f>
+        <f t="shared" si="0"/>
         <v>ATRASO</v>
       </c>
       <c r="G10" s="2">
-        <f>IF(D10&lt;=C10,0,_xlfn.DAYS(D10,C10))</f>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="H10" s="2" t="s">
@@ -2012,7 +2080,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>40</v>
       </c>
@@ -2029,11 +2097,11 @@
         <v>850</v>
       </c>
       <c r="F11" s="2" t="str">
-        <f>_xlfn.IFS(D11="","NÃO CONSTA", D11&lt;=C11,"PAGO", D11&gt;C11,"ATRASO")</f>
+        <f t="shared" si="0"/>
         <v>ATRASO</v>
       </c>
       <c r="G11" s="2">
-        <f>IF(D11&lt;=C11,0,_xlfn.DAYS(D11,C11))</f>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="H11" s="2" t="s">
@@ -2043,7 +2111,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>47</v>
       </c>
@@ -2060,11 +2128,11 @@
         <v>1047.76</v>
       </c>
       <c r="F12" s="2" t="str">
-        <f>_xlfn.IFS(D12="","NÃO CONSTA", D12&lt;=C12,"PAGO", D12&gt;C12,"ATRASO")</f>
+        <f t="shared" si="0"/>
         <v>ATRASO</v>
       </c>
       <c r="G12" s="2">
-        <f>IF(D12&lt;=C12,0,_xlfn.DAYS(D12,C12))</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="H12" s="2" t="s">
@@ -2074,7 +2142,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>48</v>
       </c>
@@ -2091,11 +2159,11 @@
         <v>1047.76</v>
       </c>
       <c r="F13" s="2" t="str">
-        <f>_xlfn.IFS(D13="","NÃO CONSTA", D13&lt;=C13,"PAGO", D13&gt;C13,"ATRASO")</f>
+        <f t="shared" si="0"/>
         <v>ATRASO</v>
       </c>
       <c r="G13" s="2">
-        <f>IF(D13&lt;=C13,0,_xlfn.DAYS(D13,C13))</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="H13" s="2" t="s">
@@ -2105,23 +2173,23 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="5">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" s="15"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="17">
         <f>SUM(E2:E13)</f>
         <v>9489.3799999999992</v>
       </c>
-      <c r="F14" s="13" t="s">
+      <c r="F14" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G14" s="19"/>
+      <c r="H14" s="19"/>
+      <c r="I14" s="19"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>17</v>
       </c>
@@ -2134,11 +2202,11 @@
       <c r="D15" s="2"/>
       <c r="E15" s="5"/>
       <c r="F15" s="2" t="str">
-        <f>_xlfn.IFS(D15="","NÃO CONSTA", D15&lt;=C15,"PAGO", D15&gt;C15,"ATRASO")</f>
+        <f t="shared" ref="F15:F22" si="2">_xlfn.IFS(D15="","NÃO CONSTA", D15&lt;=C15,"PAGO", D15&gt;C15,"ATRASO")</f>
         <v>NÃO CONSTA</v>
       </c>
       <c r="G15" s="2">
-        <f>IF(D15&lt;=C15,0,_xlfn.DAYS(D15,C15))</f>
+        <f t="shared" ref="G15:G22" si="3">IF(D15&lt;=C15,0,_xlfn.DAYS(D15,C15))</f>
         <v>0</v>
       </c>
       <c r="H15" s="2" t="s">
@@ -2148,7 +2216,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>24</v>
       </c>
@@ -2161,11 +2229,11 @@
       <c r="D16" s="2"/>
       <c r="E16" s="5"/>
       <c r="F16" s="2" t="str">
-        <f>_xlfn.IFS(D16="","NÃO CONSTA", D16&lt;=C16,"PAGO", D16&gt;C16,"ATRASO")</f>
+        <f t="shared" si="2"/>
         <v>NÃO CONSTA</v>
       </c>
       <c r="G16" s="2">
-        <f>IF(D16&lt;=C16,0,_xlfn.DAYS(D16,C16))</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H16" s="2" t="s">
@@ -2175,7 +2243,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>29</v>
       </c>
@@ -2188,11 +2256,11 @@
       <c r="D17" s="2"/>
       <c r="E17" s="5"/>
       <c r="F17" s="2" t="str">
-        <f>_xlfn.IFS(D17="","NÃO CONSTA", D17&lt;=C17,"PAGO", D17&gt;C17,"ATRASO")</f>
+        <f t="shared" si="2"/>
         <v>NÃO CONSTA</v>
       </c>
       <c r="G17" s="2">
-        <f>IF(D17&lt;=C17,0,_xlfn.DAYS(D17,C17))</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H17" s="2" t="s">
@@ -2202,7 +2270,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>33</v>
       </c>
@@ -2215,11 +2283,11 @@
       <c r="D18" s="2"/>
       <c r="E18" s="5"/>
       <c r="F18" s="2" t="str">
-        <f>_xlfn.IFS(D18="","NÃO CONSTA", D18&lt;=C18,"PAGO", D18&gt;C18,"ATRASO")</f>
+        <f t="shared" si="2"/>
         <v>NÃO CONSTA</v>
       </c>
       <c r="G18" s="2">
-        <f>IF(D18&lt;=C18,0,_xlfn.DAYS(D18,C18))</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H18" s="2" t="s">
@@ -2229,7 +2297,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>37</v>
       </c>
@@ -2242,11 +2310,11 @@
       <c r="D19" s="2"/>
       <c r="E19" s="5"/>
       <c r="F19" s="2" t="str">
-        <f>_xlfn.IFS(D19="","NÃO CONSTA", D19&lt;=C19,"PAGO", D19&gt;C19,"ATRASO")</f>
+        <f t="shared" si="2"/>
         <v>NÃO CONSTA</v>
       </c>
       <c r="G19" s="2">
-        <f>IF(D19&lt;=C19,0,_xlfn.DAYS(D19,C19))</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H19" s="2" t="s">
@@ -2256,7 +2324,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>41</v>
       </c>
@@ -2269,11 +2337,11 @@
       <c r="D20" s="2"/>
       <c r="E20" s="5"/>
       <c r="F20" s="2" t="str">
-        <f>_xlfn.IFS(D20="","NÃO CONSTA", D20&lt;=C20,"PAGO", D20&gt;C20,"ATRASO")</f>
+        <f t="shared" si="2"/>
         <v>NÃO CONSTA</v>
       </c>
       <c r="G20" s="2">
-        <f>IF(D20&lt;=C20,0,_xlfn.DAYS(D20,C20))</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H20" s="2" t="s">
@@ -2283,7 +2351,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>46</v>
       </c>
@@ -2296,11 +2364,11 @@
       <c r="D21" s="4"/>
       <c r="E21" s="5"/>
       <c r="F21" s="2" t="str">
-        <f>_xlfn.IFS(D21="","NÃO CONSTA", D21&lt;=C21,"PAGO", D21&gt;C21,"ATRASO")</f>
+        <f t="shared" si="2"/>
         <v>NÃO CONSTA</v>
       </c>
       <c r="G21" s="2">
-        <f>IF(D21&lt;=C21,0,_xlfn.DAYS(D21,C21))</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H21" s="2" t="s">
@@ -2310,7 +2378,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>49</v>
       </c>
@@ -2323,11 +2391,11 @@
       <c r="D22" s="2"/>
       <c r="E22" s="5"/>
       <c r="F22" s="2" t="str">
-        <f>_xlfn.IFS(D22="","NÃO CONSTA", D22&lt;=C22,"PAGO", D22&gt;C22,"ATRASO")</f>
+        <f t="shared" si="2"/>
         <v>NÃO CONSTA</v>
       </c>
       <c r="G22" s="2">
-        <f>IF(D22&lt;=C22,0,_xlfn.DAYS(D22,C22))</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H22" s="2" t="s">
@@ -2337,22 +2405,22 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="1"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="14">
-        <v>0</v>
-      </c>
-      <c r="F23" s="13" t="s">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A23" s="15"/>
+      <c r="B23" s="16"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="20">
+        <v>0</v>
+      </c>
+      <c r="F23" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G23" s="19"/>
+      <c r="H23" s="19"/>
+      <c r="I23" s="19"/>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>18</v>
       </c>
@@ -2369,11 +2437,11 @@
         <v>573.76</v>
       </c>
       <c r="F24" s="2" t="str">
-        <f>_xlfn.IFS(D24="","NÃO CONSTA", D24&lt;=C24,"PAGO", D24&gt;C24,"ATRASO")</f>
+        <f t="shared" ref="F24:F37" si="4">_xlfn.IFS(D24="","NÃO CONSTA", D24&lt;=C24,"PAGO", D24&gt;C24,"ATRASO")</f>
         <v>PAGO</v>
       </c>
       <c r="G24" s="2">
-        <f>IF(D24&lt;=C24,0,_xlfn.DAYS(D24,C24))</f>
+        <f t="shared" ref="G24:G37" si="5">IF(D24&lt;=C24,0,_xlfn.DAYS(D24,C24))</f>
         <v>0</v>
       </c>
       <c r="H24" s="2" t="s">
@@ -2383,7 +2451,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>19</v>
       </c>
@@ -2400,11 +2468,11 @@
         <v>582.48</v>
       </c>
       <c r="F25" s="2" t="str">
-        <f>_xlfn.IFS(D25="","NÃO CONSTA", D25&lt;=C25,"PAGO", D25&gt;C25,"ATRASO")</f>
+        <f t="shared" si="4"/>
         <v>PAGO</v>
       </c>
       <c r="G25" s="2">
-        <f>IF(D25&lt;=C25,0,_xlfn.DAYS(D25,C25))</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="H25" s="2" t="s">
@@ -2414,7 +2482,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>20</v>
       </c>
@@ -2431,11 +2499,11 @@
         <v>582.48</v>
       </c>
       <c r="F26" s="2" t="str">
-        <f>_xlfn.IFS(D26="","NÃO CONSTA", D26&lt;=C26,"PAGO", D26&gt;C26,"ATRASO")</f>
+        <f t="shared" si="4"/>
         <v>PAGO</v>
       </c>
       <c r="G26" s="2">
-        <f>IF(D26&lt;=C26,0,_xlfn.DAYS(D26,C26))</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="H26" s="2" t="s">
@@ -2445,7 +2513,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>21</v>
       </c>
@@ -2462,11 +2530,11 @@
         <v>582.88</v>
       </c>
       <c r="F27" s="2" t="str">
-        <f>_xlfn.IFS(D27="","NÃO CONSTA", D27&lt;=C27,"PAGO", D27&gt;C27,"ATRASO")</f>
+        <f t="shared" si="4"/>
         <v>PAGO</v>
       </c>
       <c r="G27" s="2">
-        <f>IF(D27&lt;=C27,0,_xlfn.DAYS(D27,C27))</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="H27" s="2" t="s">
@@ -2476,7 +2544,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>22</v>
       </c>
@@ -2493,11 +2561,11 @@
         <v>582.88</v>
       </c>
       <c r="F28" s="2" t="str">
-        <f>_xlfn.IFS(D28="","NÃO CONSTA", D28&lt;=C28,"PAGO", D28&gt;C28,"ATRASO")</f>
+        <f t="shared" si="4"/>
         <v>PAGO</v>
       </c>
       <c r="G28" s="2">
-        <f>IF(D28&lt;=C28,0,_xlfn.DAYS(D28,C28))</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="H28" s="2" t="s">
@@ -2507,7 +2575,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>31</v>
       </c>
@@ -2524,11 +2592,11 @@
         <v>765.44</v>
       </c>
       <c r="F29" s="2" t="str">
-        <f>_xlfn.IFS(D29="","NÃO CONSTA", D29&lt;=C29,"PAGO", D29&gt;C29,"ATRASO")</f>
+        <f t="shared" si="4"/>
         <v>PAGO</v>
       </c>
       <c r="G29" s="2">
-        <f>IF(D29&lt;=C29,0,_xlfn.DAYS(D29,C29))</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="H29" s="2" t="s">
@@ -2538,7 +2606,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>32</v>
       </c>
@@ -2555,11 +2623,11 @@
         <v>765.44</v>
       </c>
       <c r="F30" s="2" t="str">
-        <f>_xlfn.IFS(D30="","NÃO CONSTA", D30&lt;=C30,"PAGO", D30&gt;C30,"ATRASO")</f>
+        <f t="shared" si="4"/>
         <v>PAGO</v>
       </c>
       <c r="G30" s="2">
-        <f>IF(D30&lt;=C30,0,_xlfn.DAYS(D30,C30))</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="H30" s="2" t="s">
@@ -2569,7 +2637,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>34</v>
       </c>
@@ -2586,11 +2654,11 @@
         <v>800</v>
       </c>
       <c r="F31" s="2" t="str">
-        <f>_xlfn.IFS(D31="","NÃO CONSTA", D31&lt;=C31,"PAGO", D31&gt;C31,"ATRASO")</f>
+        <f t="shared" si="4"/>
         <v>PAGO</v>
       </c>
       <c r="G31" s="2">
-        <f>IF(D31&lt;=C31,0,_xlfn.DAYS(D31,C31))</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="H31" s="2" t="s">
@@ -2600,7 +2668,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>35</v>
       </c>
@@ -2617,11 +2685,11 @@
         <v>800</v>
       </c>
       <c r="F32" s="2" t="str">
-        <f>_xlfn.IFS(D32="","NÃO CONSTA", D32&lt;=C32,"PAGO", D32&gt;C32,"ATRASO")</f>
+        <f t="shared" si="4"/>
         <v>PAGO</v>
       </c>
       <c r="G32" s="2">
-        <f>IF(D32&lt;=C32,0,_xlfn.DAYS(D32,C32))</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="H32" s="2" t="s">
@@ -2631,7 +2699,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>42</v>
       </c>
@@ -2648,11 +2716,11 @@
         <v>931.39</v>
       </c>
       <c r="F33" s="2" t="str">
-        <f>_xlfn.IFS(D33="","NÃO CONSTA", D33&lt;=C33,"PAGO", D33&gt;C33,"ATRASO")</f>
+        <f t="shared" si="4"/>
         <v>PAGO</v>
       </c>
       <c r="G33" s="2">
-        <f>IF(D33&lt;=C33,0,_xlfn.DAYS(D33,C33))</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="H33" s="2" t="s">
@@ -2662,7 +2730,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>43</v>
       </c>
@@ -2679,11 +2747,11 @@
         <v>931.39</v>
       </c>
       <c r="F34" s="2" t="str">
-        <f>_xlfn.IFS(D34="","NÃO CONSTA", D34&lt;=C34,"PAGO", D34&gt;C34,"ATRASO")</f>
+        <f t="shared" si="4"/>
         <v>PAGO</v>
       </c>
       <c r="G34" s="2">
-        <f>IF(D34&lt;=C34,0,_xlfn.DAYS(D34,C34))</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="H34" s="2" t="s">
@@ -2693,7 +2761,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>44</v>
       </c>
@@ -2710,11 +2778,11 @@
         <v>966</v>
       </c>
       <c r="F35" s="2" t="str">
-        <f>_xlfn.IFS(D35="","NÃO CONSTA", D35&lt;=C35,"PAGO", D35&gt;C35,"ATRASO")</f>
+        <f t="shared" si="4"/>
         <v>PAGO</v>
       </c>
       <c r="G35" s="2">
-        <f>IF(D35&lt;=C35,0,_xlfn.DAYS(D35,C35))</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="H35" s="2" t="s">
@@ -2724,7 +2792,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>45</v>
       </c>
@@ -2741,11 +2809,11 @@
         <v>985.5</v>
       </c>
       <c r="F36" s="2" t="str">
-        <f>_xlfn.IFS(D36="","NÃO CONSTA", D36&lt;=C36,"PAGO", D36&gt;C36,"ATRASO")</f>
+        <f t="shared" si="4"/>
         <v>PAGO</v>
       </c>
       <c r="G36" s="2">
-        <f>IF(D36&lt;=C36,0,_xlfn.DAYS(D36,C36))</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="H36" s="2" t="s">
@@ -2755,7 +2823,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>50</v>
       </c>
@@ -2772,11 +2840,11 @@
         <v>1132</v>
       </c>
       <c r="F37" s="2" t="str">
-        <f>_xlfn.IFS(D37="","NÃO CONSTA", D37&lt;=C37,"PAGO", D37&gt;C37,"ATRASO")</f>
+        <f t="shared" si="4"/>
         <v>PAGO</v>
       </c>
       <c r="G37" s="2">
-        <f>IF(D37&lt;=C37,0,_xlfn.DAYS(D37,C37))</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="H37" s="2" t="s">
@@ -2786,35 +2854,1182 @@
         <v>9</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="1"/>
-      <c r="B38" s="4"/>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="5">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A38" s="15"/>
+      <c r="B38" s="16"/>
+      <c r="C38" s="16"/>
+      <c r="D38" s="16"/>
+      <c r="E38" s="17">
         <f>SUM(E24:E37)</f>
         <v>10981.640000000001</v>
       </c>
-      <c r="F38" s="13" t="s">
+      <c r="F38" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="G38" s="2"/>
-      <c r="H38" s="2"/>
-      <c r="I38" s="2"/>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E39" s="16">
+      <c r="G38" s="19"/>
+      <c r="H38" s="19"/>
+      <c r="I38" s="19"/>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E39" s="14">
         <f>SUM(E24:E37,E2:E13)</f>
         <v>20471.019999999997</v>
       </c>
-      <c r="F39" s="15" t="s">
+      <c r="F39" s="13" t="s">
         <v>54</v>
       </c>
     </row>
   </sheetData>
-  <sortState ref="A2:I37">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I37">
     <sortCondition ref="F2"/>
   </sortState>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60BDCD04-A9C2-4C72-B1B7-F86E7F9596CE}">
+  <dimension ref="A3:L44"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>55</v>
+      </c>
+      <c r="K3" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="L3" s="22"/>
+    </row>
+    <row r="4" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="G4" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H4" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="I4" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="K4" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="L4" s="1"/>
+    </row>
+    <row r="5" spans="1:12" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="K5" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="L5" s="1"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="K6" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="L6" s="1"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="K7" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="L7" s="1"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="K8" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="L8" s="1"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="D10" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="E10" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="F10" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="G10" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H10" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="I10" s="21" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="8">
+        <v>43191</v>
+      </c>
+      <c r="C11" s="8">
+        <v>43217</v>
+      </c>
+      <c r="D11" s="9"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="9" t="str">
+        <f>_xlfn.IFS(D11="","NÃO CONSTA", D11&lt;=C11,"PAGO", D11&gt;C11,"ATRASO")</f>
+        <v>NÃO CONSTA</v>
+      </c>
+      <c r="G11" s="2">
+        <f>IF(D11&lt;=C11,0,_xlfn.DAYS(D11,C11))</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="I11" s="9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="4">
+        <v>43191</v>
+      </c>
+      <c r="C12" s="4">
+        <v>43217</v>
+      </c>
+      <c r="D12" s="4">
+        <v>43217</v>
+      </c>
+      <c r="E12" s="5">
+        <v>573.76</v>
+      </c>
+      <c r="F12" s="9" t="str">
+        <f t="shared" ref="F12:F44" si="0">_xlfn.IFS(D12="","NÃO CONSTA", D12&lt;=C12,"PAGO", D12&gt;C12,"ATRASO")</f>
+        <v>PAGO</v>
+      </c>
+      <c r="G12" s="2">
+        <f>IF(D12&lt;=C12,0,_xlfn.DAYS(D12,C12))</f>
+        <v>0</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="4">
+        <v>43193</v>
+      </c>
+      <c r="C13" s="4">
+        <v>43218</v>
+      </c>
+      <c r="D13" s="4">
+        <v>43218</v>
+      </c>
+      <c r="E13" s="5">
+        <v>582.48</v>
+      </c>
+      <c r="F13" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>PAGO</v>
+      </c>
+      <c r="G13" s="2">
+        <f t="shared" ref="G13:G44" si="1">IF(D13&lt;=C13,0,_xlfn.DAYS(D13,C13))</f>
+        <v>0</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="4">
+        <v>43193</v>
+      </c>
+      <c r="C14" s="4">
+        <v>43218</v>
+      </c>
+      <c r="D14" s="4">
+        <v>43218</v>
+      </c>
+      <c r="E14" s="5">
+        <v>582.48</v>
+      </c>
+      <c r="F14" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>PAGO</v>
+      </c>
+      <c r="G14" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="4">
+        <v>43191</v>
+      </c>
+      <c r="C15" s="4">
+        <v>43219</v>
+      </c>
+      <c r="D15" s="4">
+        <v>43219</v>
+      </c>
+      <c r="E15" s="5">
+        <v>582.88</v>
+      </c>
+      <c r="F15" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>PAGO</v>
+      </c>
+      <c r="G15" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="4">
+        <v>43191</v>
+      </c>
+      <c r="C16" s="4">
+        <v>43219</v>
+      </c>
+      <c r="D16" s="4">
+        <v>43219</v>
+      </c>
+      <c r="E16" s="5">
+        <v>582.88</v>
+      </c>
+      <c r="F16" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>PAGO</v>
+      </c>
+      <c r="G16" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="4">
+        <v>43191</v>
+      </c>
+      <c r="C17" s="4">
+        <v>43221</v>
+      </c>
+      <c r="D17" s="4">
+        <v>43222</v>
+      </c>
+      <c r="E17" s="5">
+        <v>611.82000000000005</v>
+      </c>
+      <c r="F17" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>ATRASO</v>
+      </c>
+      <c r="G17" s="2">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" s="4">
+        <v>43191</v>
+      </c>
+      <c r="C18" s="4">
+        <v>43221</v>
+      </c>
+      <c r="D18" s="2"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>NÃO CONSTA</v>
+      </c>
+      <c r="G18" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="4">
+        <v>43193</v>
+      </c>
+      <c r="C19" s="4">
+        <v>43219</v>
+      </c>
+      <c r="D19" s="4">
+        <v>43220</v>
+      </c>
+      <c r="E19" s="5">
+        <v>633.63</v>
+      </c>
+      <c r="F19" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>ATRASO</v>
+      </c>
+      <c r="G19" s="2">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="4">
+        <v>43193</v>
+      </c>
+      <c r="C20" s="4">
+        <v>43219</v>
+      </c>
+      <c r="D20" s="4">
+        <v>43220</v>
+      </c>
+      <c r="E20" s="5">
+        <v>633.63</v>
+      </c>
+      <c r="F20" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>ATRASO</v>
+      </c>
+      <c r="G20" s="2">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" s="4">
+        <v>43191</v>
+      </c>
+      <c r="C21" s="4">
+        <v>43212</v>
+      </c>
+      <c r="D21" s="4">
+        <v>43213</v>
+      </c>
+      <c r="E21" s="5">
+        <v>700</v>
+      </c>
+      <c r="F21" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>ATRASO</v>
+      </c>
+      <c r="G21" s="2">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B22" s="4">
+        <v>43191</v>
+      </c>
+      <c r="C22" s="4">
+        <v>43213</v>
+      </c>
+      <c r="D22" s="4">
+        <v>43214</v>
+      </c>
+      <c r="E22" s="5">
+        <v>733.37</v>
+      </c>
+      <c r="F22" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>ATRASO</v>
+      </c>
+      <c r="G22" s="2">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B23" s="4">
+        <v>43193</v>
+      </c>
+      <c r="C23" s="4">
+        <v>43221</v>
+      </c>
+      <c r="D23" s="2"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>NÃO CONSTA</v>
+      </c>
+      <c r="G23" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24" s="4">
+        <v>43193</v>
+      </c>
+      <c r="C24" s="4">
+        <v>43221</v>
+      </c>
+      <c r="D24" s="4">
+        <v>43222</v>
+      </c>
+      <c r="E24" s="5">
+        <v>733.37</v>
+      </c>
+      <c r="F24" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>ATRASO</v>
+      </c>
+      <c r="G24" s="2">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A25" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B25" s="4">
+        <v>43193</v>
+      </c>
+      <c r="C25" s="4">
+        <v>43223</v>
+      </c>
+      <c r="D25" s="4">
+        <v>43221</v>
+      </c>
+      <c r="E25" s="5">
+        <v>765.44</v>
+      </c>
+      <c r="F25" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>PAGO</v>
+      </c>
+      <c r="G25" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" s="4">
+        <v>43193</v>
+      </c>
+      <c r="C26" s="4">
+        <v>43223</v>
+      </c>
+      <c r="D26" s="4">
+        <v>43221</v>
+      </c>
+      <c r="E26" s="5">
+        <v>765.44</v>
+      </c>
+      <c r="F26" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>PAGO</v>
+      </c>
+      <c r="G26" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B27" s="4">
+        <v>43191</v>
+      </c>
+      <c r="C27" s="4">
+        <v>43214</v>
+      </c>
+      <c r="D27" s="2"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>NÃO CONSTA</v>
+      </c>
+      <c r="G27" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B28" s="4">
+        <v>43191</v>
+      </c>
+      <c r="C28" s="4">
+        <v>43216</v>
+      </c>
+      <c r="D28" s="4">
+        <v>43214</v>
+      </c>
+      <c r="E28" s="5">
+        <v>800</v>
+      </c>
+      <c r="F28" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>PAGO</v>
+      </c>
+      <c r="G28" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A29" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B29" s="4">
+        <v>43191</v>
+      </c>
+      <c r="C29" s="4">
+        <v>43216</v>
+      </c>
+      <c r="D29" s="4">
+        <v>43214</v>
+      </c>
+      <c r="E29" s="5">
+        <v>800</v>
+      </c>
+      <c r="F29" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>PAGO</v>
+      </c>
+      <c r="G29" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A30" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B30" s="4">
+        <v>43194</v>
+      </c>
+      <c r="C30" s="4">
+        <v>43217</v>
+      </c>
+      <c r="D30" s="4">
+        <v>43227</v>
+      </c>
+      <c r="E30" s="5">
+        <v>815.3</v>
+      </c>
+      <c r="F30" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>ATRASO</v>
+      </c>
+      <c r="G30" s="2">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B31" s="4">
+        <v>43194</v>
+      </c>
+      <c r="C31" s="4">
+        <v>43217</v>
+      </c>
+      <c r="D31" s="2"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>NÃO CONSTA</v>
+      </c>
+      <c r="G31" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A32" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B32" s="4">
+        <v>43191</v>
+      </c>
+      <c r="C32" s="4">
+        <v>43217</v>
+      </c>
+      <c r="D32" s="4">
+        <v>43227</v>
+      </c>
+      <c r="E32" s="5">
+        <v>841.37</v>
+      </c>
+      <c r="F32" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>ATRASO</v>
+      </c>
+      <c r="G32" s="2">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B33" s="4">
+        <v>43191</v>
+      </c>
+      <c r="C33" s="4">
+        <v>43217</v>
+      </c>
+      <c r="D33" s="4">
+        <v>43227</v>
+      </c>
+      <c r="E33" s="5">
+        <v>841.37</v>
+      </c>
+      <c r="F33" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>ATRASO</v>
+      </c>
+      <c r="G33" s="2">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B34" s="4">
+        <v>43193</v>
+      </c>
+      <c r="C34" s="4">
+        <v>43214</v>
+      </c>
+      <c r="D34" s="4">
+        <v>43224</v>
+      </c>
+      <c r="E34" s="5">
+        <v>850</v>
+      </c>
+      <c r="F34" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>ATRASO</v>
+      </c>
+      <c r="G34" s="2">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B35" s="4">
+        <v>43193</v>
+      </c>
+      <c r="C35" s="4">
+        <v>43214</v>
+      </c>
+      <c r="D35" s="2"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>NÃO CONSTA</v>
+      </c>
+      <c r="G35" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A36" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B36" s="4">
+        <v>43193</v>
+      </c>
+      <c r="C36" s="4">
+        <v>43215</v>
+      </c>
+      <c r="D36" s="4">
+        <v>43212</v>
+      </c>
+      <c r="E36" s="5">
+        <v>931.39</v>
+      </c>
+      <c r="F36" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>PAGO</v>
+      </c>
+      <c r="G36" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A37" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B37" s="4">
+        <v>43193</v>
+      </c>
+      <c r="C37" s="4">
+        <v>43215</v>
+      </c>
+      <c r="D37" s="4">
+        <v>43212</v>
+      </c>
+      <c r="E37" s="5">
+        <v>931.39</v>
+      </c>
+      <c r="F37" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>PAGO</v>
+      </c>
+      <c r="G37" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A38" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B38" s="4">
+        <v>43193</v>
+      </c>
+      <c r="C38" s="4">
+        <v>43216</v>
+      </c>
+      <c r="D38" s="4">
+        <v>43213</v>
+      </c>
+      <c r="E38" s="5">
+        <v>966</v>
+      </c>
+      <c r="F38" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>PAGO</v>
+      </c>
+      <c r="G38" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A39" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B39" s="4">
+        <v>43193</v>
+      </c>
+      <c r="C39" s="4">
+        <v>43218</v>
+      </c>
+      <c r="D39" s="4">
+        <v>43215</v>
+      </c>
+      <c r="E39" s="5">
+        <v>985.5</v>
+      </c>
+      <c r="F39" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>PAGO</v>
+      </c>
+      <c r="G39" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A40" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B40" s="4">
+        <v>43193</v>
+      </c>
+      <c r="C40" s="4">
+        <v>43218</v>
+      </c>
+      <c r="D40" s="4"/>
+      <c r="E40" s="5"/>
+      <c r="F40" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>NÃO CONSTA</v>
+      </c>
+      <c r="G40" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B41" s="4">
+        <v>43193</v>
+      </c>
+      <c r="C41" s="4">
+        <v>43219</v>
+      </c>
+      <c r="D41" s="4">
+        <v>43224</v>
+      </c>
+      <c r="E41" s="5">
+        <v>1047.76</v>
+      </c>
+      <c r="F41" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>ATRASO</v>
+      </c>
+      <c r="G41" s="2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B42" s="4">
+        <v>43193</v>
+      </c>
+      <c r="C42" s="4">
+        <v>43219</v>
+      </c>
+      <c r="D42" s="4">
+        <v>43224</v>
+      </c>
+      <c r="E42" s="5">
+        <v>1047.76</v>
+      </c>
+      <c r="F42" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>ATRASO</v>
+      </c>
+      <c r="G42" s="2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A43" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B43" s="4">
+        <v>43191</v>
+      </c>
+      <c r="C43" s="4">
+        <v>43219</v>
+      </c>
+      <c r="D43" s="2"/>
+      <c r="E43" s="5"/>
+      <c r="F43" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>NÃO CONSTA</v>
+      </c>
+      <c r="G43" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A44" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B44" s="4">
+        <v>43191</v>
+      </c>
+      <c r="C44" s="4">
+        <v>43219</v>
+      </c>
+      <c r="D44" s="4">
+        <v>43219</v>
+      </c>
+      <c r="E44" s="5">
+        <v>1132</v>
+      </c>
+      <c r="F44" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>PAGO</v>
+      </c>
+      <c r="G44" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="K3:L3"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>